<commit_message>
Remove xlsx dependency, parse Excel natively
</commit_message>
<xml_diff>
--- a/estimator.xlsx
+++ b/estimator.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="83">
   <si>
     <t>Customer:</t>
   </si>
@@ -267,6 +267,9 @@
   </si>
   <si>
     <t>Notes:</t>
+  </si>
+  <si>
+    <t>8109-600</t>
   </si>
   <si>
     <t>60Hp VFD</t>
@@ -6340,14 +6343,14 @@
       <c r="A276" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B276" s="1">
-        <v>8109</v>
+      <c r="B276" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="C276" s="1">
         <v>1</v>
       </c>
       <c r="D276" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F276" s="1">
         <v>12</v>

</xml_diff>